<commit_message>
Hora no abastecimento, situacao enxuta e cadastro de abastecedores
- campo Hora no lancamento, ja preenchido com a hora atual e editavel;
  aparece nos recentes e em Corrigir Dados, e vai para a planilha numa
  coluna Hora (sync, Codigo.gs e o modelo da Diretoria)
- Situacao do equipamento passa a ter so Operando e Manutencao;
  statusDaSituacao continua entendendo os textos antigos, senao os
  lancamentos ja gravados mudariam de status no Painel e na Frota
- tela Operadores ganha o cadastro de Abastecedores (adicionar e apagar),
  sem mexer no historico de quem ja abasteceu
- versao r34

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zdUaDFEZQ75SJ6DGMruWx
</commit_message>
<xml_diff>
--- a/google-sheets/GP2T-Planilha-Diretoria.xlsx
+++ b/google-sheets/GP2T-Planilha-Diretoria.xlsx
@@ -1839,25 +1839,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1882,75 +1883,80 @@
       </c>
       <c r="B3" s="30" t="inlineStr">
         <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
           <t>Equipamento</t>
         </is>
       </c>
-      <c r="C3" s="30" t="inlineStr">
+      <c r="D3" s="30" t="inlineStr">
         <is>
           <t>Operador</t>
         </is>
       </c>
-      <c r="D3" s="30" t="inlineStr">
+      <c r="E3" s="30" t="inlineStr">
         <is>
           <t>Horímetro Inicial</t>
         </is>
       </c>
-      <c r="E3" s="30" t="inlineStr">
+      <c r="F3" s="30" t="inlineStr">
         <is>
           <t>Horímetro Final</t>
         </is>
       </c>
-      <c r="F3" s="30" t="inlineStr">
+      <c r="G3" s="30" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
       </c>
-      <c r="G3" s="30" t="inlineStr">
+      <c r="H3" s="30" t="inlineStr">
         <is>
           <t>Litros</t>
         </is>
       </c>
-      <c r="H3" s="30" t="inlineStr">
+      <c r="I3" s="30" t="inlineStr">
         <is>
           <t>Combustível</t>
         </is>
       </c>
-      <c r="I3" s="30" t="inlineStr">
+      <c r="J3" s="30" t="inlineStr">
         <is>
           <t>ARLA (L)</t>
         </is>
       </c>
-      <c r="J3" s="30" t="inlineStr">
+      <c r="K3" s="30" t="inlineStr">
         <is>
           <t>KM Rodado</t>
         </is>
       </c>
-      <c r="K3" s="30" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="L3" s="30" t="inlineStr">
+      <c r="M3" s="30" t="inlineStr">
         <is>
           <t>Unidade</t>
         </is>
       </c>
-      <c r="M3" s="30" t="inlineStr">
+      <c r="N3" s="30" t="inlineStr">
         <is>
           <t>Toneladas</t>
         </is>
       </c>
-      <c r="N3" s="30" t="inlineStr">
+      <c r="O3" s="30" t="inlineStr">
         <is>
           <t>L/Ton</t>
         </is>
       </c>
-      <c r="O3" s="30" t="inlineStr">
+      <c r="P3" s="30" t="inlineStr">
         <is>
           <t>Situação</t>
         </is>
       </c>
-      <c r="P3" s="30" t="inlineStr">
+      <c r="Q3" s="30" t="inlineStr">
         <is>
           <t>_id</t>
         </is>

</xml_diff>